<commit_message>
vault backup: 2026-04-15 10:46:16
</commit_message>
<xml_diff>
--- a/work/项目/运营Uplift模型/运营uplift模型现状分析和规划.xlsx
+++ b/work/项目/运营Uplift模型/运营uplift模型现状分析和规划.xlsx
@@ -957,7 +957,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1085,6 +1085,17 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="35" fillId="46" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="42" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="44" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="45" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1678,7 +1689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H77"/>
+  <dimension ref="A1:I77"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.23076923076923" defaultRowHeight="16.8"/>
   <cols>
     <col width="3" customWidth="1" style="4" min="1" max="1"/>
@@ -1689,6 +1700,7 @@
     <col width="18" customWidth="1" style="4" min="6" max="6"/>
     <col width="22" customWidth="1" style="4" min="7" max="7"/>
     <col width="3" customWidth="1" style="4" min="8" max="8"/>
+    <col width="20" customWidth="1" style="4" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1748,15 +1760,15 @@
     <row r="7" ht="22" customHeight="1" s="4">
       <c r="A7" s="32" t="n"/>
       <c r="B7" s="32" t="n"/>
-      <c r="C7" s="44" t="inlineStr">
+      <c r="C7" s="35" t="inlineStr">
         <is>
           <t>实验基本情况</t>
         </is>
       </c>
-      <c r="D7" s="45" t="n"/>
-      <c r="E7" s="45" t="n"/>
-      <c r="F7" s="45" t="n"/>
-      <c r="G7" s="46" t="n"/>
+      <c r="D7" s="51" t="n"/>
+      <c r="E7" s="51" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="52" t="n"/>
       <c r="H7" s="32" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1" s="4">
@@ -1767,14 +1779,14 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="D8" s="47" t="inlineStr">
+      <c r="D8" s="36" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="E8" s="45" t="n"/>
-      <c r="F8" s="45" t="n"/>
-      <c r="G8" s="46" t="n"/>
+      <c r="E8" s="51" t="n"/>
+      <c r="F8" s="51" t="n"/>
+      <c r="G8" s="52" t="n"/>
       <c r="H8" s="32" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1" s="4">
@@ -1785,14 +1797,14 @@
           <t>实验名称</t>
         </is>
       </c>
-      <c r="D9" s="48" t="inlineStr">
+      <c r="D9" s="38" t="inlineStr">
         <is>
           <t>续借月维度-常规-WA泳道-触达-26-长期实验-3天1次推全-0319重开（实验13248）</t>
         </is>
       </c>
-      <c r="E9" s="45" t="n"/>
-      <c r="F9" s="45" t="n"/>
-      <c r="G9" s="46" t="n"/>
+      <c r="E9" s="51" t="n"/>
+      <c r="F9" s="51" t="n"/>
+      <c r="G9" s="52" t="n"/>
       <c r="H9" s="32" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1" s="4">
@@ -1803,14 +1815,14 @@
           <t>样本规模</t>
         </is>
       </c>
-      <c r="D10" s="48" t="inlineStr">
+      <c r="D10" s="38" t="inlineStr">
         <is>
           <t>样本量190w，人维度30w+；实验组344,129人 / 对照组38,140人（比约9:1）</t>
         </is>
       </c>
-      <c r="E10" s="45" t="n"/>
-      <c r="F10" s="45" t="n"/>
-      <c r="G10" s="46" t="n"/>
+      <c r="E10" s="51" t="n"/>
+      <c r="F10" s="51" t="n"/>
+      <c r="G10" s="52" t="n"/>
       <c r="H10" s="32" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1" s="4">
@@ -1821,14 +1833,14 @@
           <t>观测指标</t>
         </is>
       </c>
-      <c r="D11" s="48" t="inlineStr">
+      <c r="D11" s="38" t="inlineStr">
         <is>
           <t>T+1放款率约2.5%，T+1信号 Spearman ρ 通过显著性检验</t>
         </is>
       </c>
-      <c r="E11" s="45" t="n"/>
-      <c r="F11" s="45" t="n"/>
-      <c r="G11" s="46" t="n"/>
+      <c r="E11" s="51" t="n"/>
+      <c r="F11" s="51" t="n"/>
+      <c r="G11" s="52" t="n"/>
       <c r="H11" s="32" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1" s="4">
@@ -1844,15 +1856,15 @@
     <row r="13" ht="22" customHeight="1" s="4">
       <c r="A13" s="32" t="n"/>
       <c r="B13" s="32" t="n"/>
-      <c r="C13" s="44" t="inlineStr">
+      <c r="C13" s="35" t="inlineStr">
         <is>
           <t>建模方案</t>
         </is>
       </c>
-      <c r="D13" s="45" t="n"/>
-      <c r="E13" s="45" t="n"/>
-      <c r="F13" s="45" t="n"/>
-      <c r="G13" s="46" t="n"/>
+      <c r="D13" s="51" t="n"/>
+      <c r="E13" s="51" t="n"/>
+      <c r="F13" s="51" t="n"/>
+      <c r="G13" s="52" t="n"/>
       <c r="H13" s="32" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1" s="4">
@@ -1863,14 +1875,14 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="D14" s="47" t="inlineStr">
+      <c r="D14" s="36" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="E14" s="45" t="n"/>
-      <c r="F14" s="45" t="n"/>
-      <c r="G14" s="46" t="n"/>
+      <c r="E14" s="51" t="n"/>
+      <c r="F14" s="51" t="n"/>
+      <c r="G14" s="52" t="n"/>
       <c r="H14" s="32" t="n"/>
     </row>
     <row r="15" ht="30" customHeight="1" s="4">
@@ -1881,14 +1893,14 @@
           <t>方法</t>
         </is>
       </c>
-      <c r="D15" s="48" t="inlineStr">
+      <c r="D15" s="38" t="inlineStr">
         <is>
           <t>基于 LGB 的 T-learner（快速基线）/ X-learner（精度更高），样本不均衡时辅以权重修正（实验:对照≈9:1）</t>
         </is>
       </c>
-      <c r="E15" s="45" t="n"/>
-      <c r="F15" s="45" t="n"/>
-      <c r="G15" s="46" t="n"/>
+      <c r="E15" s="51" t="n"/>
+      <c r="F15" s="51" t="n"/>
+      <c r="G15" s="52" t="n"/>
       <c r="H15" s="32" t="n"/>
     </row>
     <row r="16" ht="22" customHeight="1" s="4">
@@ -1899,14 +1911,14 @@
           <t>Y变量</t>
         </is>
       </c>
-      <c r="D16" s="48" t="inlineStr">
+      <c r="D16" s="38" t="inlineStr">
         <is>
           <t>T+1放款标签（0/1），辅以放款金额加权，避免选出小额下单用户</t>
         </is>
       </c>
-      <c r="E16" s="45" t="n"/>
-      <c r="F16" s="45" t="n"/>
-      <c r="G16" s="46" t="n"/>
+      <c r="E16" s="51" t="n"/>
+      <c r="F16" s="51" t="n"/>
+      <c r="G16" s="52" t="n"/>
       <c r="H16" s="32" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1" s="4">
@@ -1917,14 +1929,14 @@
           <t>特征来源</t>
         </is>
       </c>
-      <c r="D17" s="48" t="inlineStr">
+      <c r="D17" s="38" t="inlineStr">
         <is>
           <t>复贷循环贷特征，结合泳道数据特征预筛</t>
         </is>
       </c>
-      <c r="E17" s="45" t="n"/>
-      <c r="F17" s="45" t="n"/>
-      <c r="G17" s="46" t="n"/>
+      <c r="E17" s="51" t="n"/>
+      <c r="F17" s="51" t="n"/>
+      <c r="G17" s="52" t="n"/>
       <c r="H17" s="32" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1" s="4">
@@ -1935,14 +1947,14 @@
           <t>对比基准</t>
         </is>
       </c>
-      <c r="D18" s="48" t="inlineStr">
+      <c r="D18" s="38" t="inlineStr">
         <is>
           <t>回溯旧版uplift模型分作为baseline，与新模型进行Qini/AUUC对比评估</t>
         </is>
       </c>
-      <c r="E18" s="45" t="n"/>
-      <c r="F18" s="45" t="n"/>
-      <c r="G18" s="46" t="n"/>
+      <c r="E18" s="51" t="n"/>
+      <c r="F18" s="51" t="n"/>
+      <c r="G18" s="52" t="n"/>
       <c r="H18" s="32" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1" s="4">
@@ -1996,15 +2008,15 @@
     <row r="24" ht="22" customHeight="1" s="4">
       <c r="A24" s="32" t="n"/>
       <c r="B24" s="32" t="n"/>
-      <c r="C24" s="44" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>实验设计规范</t>
         </is>
       </c>
-      <c r="D24" s="45" t="n"/>
-      <c r="E24" s="45" t="n"/>
-      <c r="F24" s="45" t="n"/>
-      <c r="G24" s="46" t="n"/>
+      <c r="D24" s="51" t="n"/>
+      <c r="E24" s="51" t="n"/>
+      <c r="F24" s="51" t="n"/>
+      <c r="G24" s="52" t="n"/>
       <c r="H24" s="32" t="n"/>
     </row>
     <row r="25" ht="20" customHeight="1" s="4">
@@ -2015,14 +2027,14 @@
           <t>设计要素</t>
         </is>
       </c>
-      <c r="D25" s="47" t="inlineStr">
+      <c r="D25" s="36" t="inlineStr">
         <is>
           <t>规格</t>
         </is>
       </c>
-      <c r="E25" s="45" t="n"/>
-      <c r="F25" s="45" t="n"/>
-      <c r="G25" s="46" t="n"/>
+      <c r="E25" s="51" t="n"/>
+      <c r="F25" s="51" t="n"/>
+      <c r="G25" s="52" t="n"/>
       <c r="H25" s="32" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1" s="4">
@@ -2033,14 +2045,14 @@
           <t>实验名称</t>
         </is>
       </c>
-      <c r="D26" s="48" t="inlineStr">
+      <c r="D26" s="38" t="inlineStr">
         <is>
           <t>复贷结清/续借-纯跑批WA-干净实验（2026H2）</t>
         </is>
       </c>
-      <c r="E26" s="45" t="n"/>
-      <c r="F26" s="45" t="n"/>
-      <c r="G26" s="46" t="n"/>
+      <c r="E26" s="51" t="n"/>
+      <c r="F26" s="51" t="n"/>
+      <c r="G26" s="52" t="n"/>
       <c r="H26" s="32" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1" s="4">
@@ -2051,14 +2063,14 @@
           <t>触达方式</t>
         </is>
       </c>
-      <c r="D27" s="48" t="inlineStr">
+      <c r="D27" s="38" t="inlineStr">
         <is>
           <t>仅离线跑批WA，不含实时触达</t>
         </is>
       </c>
-      <c r="E27" s="45" t="n"/>
-      <c r="F27" s="45" t="n"/>
-      <c r="G27" s="46" t="n"/>
+      <c r="E27" s="51" t="n"/>
+      <c r="F27" s="51" t="n"/>
+      <c r="G27" s="52" t="n"/>
       <c r="H27" s="32" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1" s="4">
@@ -2069,14 +2081,14 @@
           <t>分流比例</t>
         </is>
       </c>
-      <c r="D28" s="48" t="inlineStr">
+      <c r="D28" s="38" t="inlineStr">
         <is>
           <t>实验组15% + 对照组15%</t>
         </is>
       </c>
-      <c r="E28" s="45" t="n"/>
-      <c r="F28" s="45" t="n"/>
-      <c r="G28" s="46" t="n"/>
+      <c r="E28" s="51" t="n"/>
+      <c r="F28" s="51" t="n"/>
+      <c r="G28" s="52" t="n"/>
       <c r="H28" s="32" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1" s="4">
@@ -2087,14 +2099,14 @@
           <t>互斥范围</t>
         </is>
       </c>
-      <c r="D29" s="48" t="inlineStr">
+      <c r="D29" s="38" t="inlineStr">
         <is>
           <t>与 13248、13036、12692、12912 全部互斥</t>
         </is>
       </c>
-      <c r="E29" s="45" t="n"/>
-      <c r="F29" s="45" t="n"/>
-      <c r="G29" s="46" t="n"/>
+      <c r="E29" s="51" t="n"/>
+      <c r="F29" s="51" t="n"/>
+      <c r="G29" s="52" t="n"/>
       <c r="H29" s="32" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1" s="4">
@@ -2105,14 +2117,14 @@
           <t>观测窗口</t>
         </is>
       </c>
-      <c r="D30" s="48" t="inlineStr">
+      <c r="D30" s="38" t="inlineStr">
         <is>
           <t>T+3（主）、T+7（辅助验证）</t>
         </is>
       </c>
-      <c r="E30" s="45" t="n"/>
-      <c r="F30" s="45" t="n"/>
-      <c r="G30" s="46" t="n"/>
+      <c r="E30" s="51" t="n"/>
+      <c r="F30" s="51" t="n"/>
+      <c r="G30" s="52" t="n"/>
       <c r="H30" s="32" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1" s="4">
@@ -2123,14 +2135,14 @@
           <t>启动时间</t>
         </is>
       </c>
-      <c r="D31" s="48" t="inlineStr">
+      <c r="D31" s="38" t="inlineStr">
         <is>
           <t>2026年4月下旬（待AB平台配置完成）</t>
         </is>
       </c>
-      <c r="E31" s="45" t="n"/>
-      <c r="F31" s="45" t="n"/>
-      <c r="G31" s="46" t="n"/>
+      <c r="E31" s="51" t="n"/>
+      <c r="F31" s="51" t="n"/>
+      <c r="G31" s="52" t="n"/>
       <c r="H31" s="32" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1" s="4">
@@ -2141,14 +2153,14 @@
           <t>达量时间</t>
         </is>
       </c>
-      <c r="D32" s="48" t="inlineStr">
+      <c r="D32" s="38" t="inlineStr">
         <is>
           <t>预计2026年7月</t>
         </is>
       </c>
-      <c r="E32" s="45" t="n"/>
-      <c r="F32" s="45" t="n"/>
-      <c r="G32" s="46" t="n"/>
+      <c r="E32" s="51" t="n"/>
+      <c r="F32" s="51" t="n"/>
+      <c r="G32" s="52" t="n"/>
       <c r="H32" s="32" t="n"/>
     </row>
     <row r="33" ht="18.5" customHeight="1" s="4">
@@ -2164,15 +2176,15 @@
     <row r="34" ht="22" customHeight="1" s="4">
       <c r="A34" s="32" t="n"/>
       <c r="B34" s="32" t="n"/>
-      <c r="C34" s="44" t="inlineStr">
+      <c r="C34" s="35" t="inlineStr">
         <is>
           <t>模型训练设计</t>
         </is>
       </c>
-      <c r="D34" s="45" t="n"/>
-      <c r="E34" s="45" t="n"/>
-      <c r="F34" s="45" t="n"/>
-      <c r="G34" s="46" t="n"/>
+      <c r="D34" s="51" t="n"/>
+      <c r="E34" s="51" t="n"/>
+      <c r="F34" s="51" t="n"/>
+      <c r="G34" s="52" t="n"/>
       <c r="H34" s="32" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1" s="4">
@@ -2183,14 +2195,14 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="D35" s="47" t="inlineStr">
+      <c r="D35" s="36" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="E35" s="45" t="n"/>
-      <c r="F35" s="45" t="n"/>
-      <c r="G35" s="46" t="n"/>
+      <c r="E35" s="51" t="n"/>
+      <c r="F35" s="51" t="n"/>
+      <c r="G35" s="52" t="n"/>
       <c r="H35" s="32" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1" s="4">
@@ -2201,14 +2213,14 @@
           <t>建模方法</t>
         </is>
       </c>
-      <c r="D36" s="48" t="inlineStr">
+      <c r="D36" s="38" t="inlineStr">
         <is>
           <t>S-learner（简单）/ T-learner（精度更高）/ X-learner（样本不均衡时更稳健）</t>
         </is>
       </c>
-      <c r="E36" s="45" t="n"/>
-      <c r="F36" s="45" t="n"/>
-      <c r="G36" s="46" t="n"/>
+      <c r="E36" s="51" t="n"/>
+      <c r="F36" s="51" t="n"/>
+      <c r="G36" s="52" t="n"/>
       <c r="H36" s="32" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1" s="4">
@@ -2219,14 +2231,14 @@
           <t>Y变量</t>
         </is>
       </c>
-      <c r="D37" s="48" t="inlineStr">
+      <c r="D37" s="38" t="inlineStr">
         <is>
           <t>T+1放款标签（0/1），辅以放款金额加权</t>
         </is>
       </c>
-      <c r="E37" s="45" t="n"/>
-      <c r="F37" s="45" t="n"/>
-      <c r="G37" s="46" t="n"/>
+      <c r="E37" s="51" t="n"/>
+      <c r="F37" s="51" t="n"/>
+      <c r="G37" s="52" t="n"/>
       <c r="H37" s="32" t="n"/>
     </row>
     <row r="38" ht="28" customHeight="1" s="4">
@@ -2237,14 +2249,14 @@
           <t>质量保证</t>
         </is>
       </c>
-      <c r="D38" s="48" t="inlineStr">
+      <c r="D38" s="38" t="inlineStr">
         <is>
           <t>实验/对照组均来自干净实验，ATE理论无偏；定期污染率核查（目标 &lt;5%）</t>
         </is>
       </c>
-      <c r="E38" s="45" t="n"/>
-      <c r="F38" s="45" t="n"/>
-      <c r="G38" s="46" t="n"/>
+      <c r="E38" s="51" t="n"/>
+      <c r="F38" s="51" t="n"/>
+      <c r="G38" s="52" t="n"/>
       <c r="H38" s="32" t="n"/>
     </row>
     <row r="39" ht="17.6" customHeight="1" s="4">
@@ -2278,15 +2290,15 @@
     <row r="42" ht="22" customHeight="1" s="4">
       <c r="A42" s="32" t="n"/>
       <c r="B42" s="32" t="n"/>
-      <c r="C42" s="44" t="inlineStr">
+      <c r="C42" s="35" t="inlineStr">
         <is>
           <t>进度概况</t>
         </is>
       </c>
-      <c r="D42" s="45" t="n"/>
-      <c r="E42" s="45" t="n"/>
-      <c r="F42" s="45" t="n"/>
-      <c r="G42" s="46" t="n"/>
+      <c r="D42" s="51" t="n"/>
+      <c r="E42" s="51" t="n"/>
+      <c r="F42" s="51" t="n"/>
+      <c r="G42" s="52" t="n"/>
       <c r="H42" s="32" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1" s="4">
@@ -2297,14 +2309,14 @@
           <t>项目</t>
         </is>
       </c>
-      <c r="D43" s="47" t="inlineStr">
+      <c r="D43" s="36" t="inlineStr">
         <is>
           <t>内容</t>
         </is>
       </c>
-      <c r="E43" s="45" t="n"/>
-      <c r="F43" s="45" t="n"/>
-      <c r="G43" s="46" t="n"/>
+      <c r="E43" s="51" t="n"/>
+      <c r="F43" s="51" t="n"/>
+      <c r="G43" s="52" t="n"/>
       <c r="H43" s="32" t="n"/>
     </row>
     <row r="44" ht="22" customHeight="1" s="4">
@@ -2315,14 +2327,14 @@
           <t>决策</t>
         </is>
       </c>
-      <c r="D44" s="48" t="inlineStr">
+      <c r="D44" s="38" t="inlineStr">
         <is>
           <t>与策略共同决定：模型侧评估旧版uplift模型，并使用现有数据快速训练一个模型作为对比。</t>
         </is>
       </c>
-      <c r="E44" s="45" t="n"/>
-      <c r="F44" s="45" t="n"/>
-      <c r="G44" s="46" t="n"/>
+      <c r="E44" s="51" t="n"/>
+      <c r="F44" s="51" t="n"/>
+      <c r="G44" s="52" t="n"/>
       <c r="H44" s="32" t="n"/>
     </row>
     <row r="45" ht="28" customHeight="1" s="4">
@@ -2333,14 +2345,14 @@
           <t>训练样本</t>
         </is>
       </c>
-      <c r="D45" s="48" t="inlineStr">
+      <c r="D45" s="38" t="inlineStr">
         <is>
           <t>实验13248，样本量190w（人维度30w+），当前仅有的离线跑批实验样本。</t>
         </is>
       </c>
-      <c r="E45" s="45" t="n"/>
-      <c r="F45" s="45" t="n"/>
-      <c r="G45" s="46" t="n"/>
+      <c r="E45" s="51" t="n"/>
+      <c r="F45" s="51" t="n"/>
+      <c r="G45" s="52" t="n"/>
       <c r="H45" s="32" t="n"/>
     </row>
     <row r="46" ht="34" customHeight="1" s="4">
@@ -2374,15 +2386,15 @@
     <row r="49" ht="22" customHeight="1" s="4">
       <c r="A49" s="32" t="n"/>
       <c r="B49" s="32" t="n"/>
-      <c r="C49" s="44" t="inlineStr">
+      <c r="C49" s="35" t="inlineStr">
         <is>
           <t>待办事项</t>
         </is>
       </c>
-      <c r="D49" s="45" t="n"/>
-      <c r="E49" s="45" t="n"/>
-      <c r="F49" s="45" t="n"/>
-      <c r="G49" s="46" t="n"/>
+      <c r="D49" s="51" t="n"/>
+      <c r="E49" s="51" t="n"/>
+      <c r="F49" s="51" t="n"/>
+      <c r="G49" s="52" t="n"/>
       <c r="H49" s="32" t="n"/>
     </row>
     <row r="50" ht="20" customHeight="1" s="4">
@@ -2393,14 +2405,14 @@
           <t>#</t>
         </is>
       </c>
-      <c r="D50" s="47" t="inlineStr">
+      <c r="D50" s="36" t="inlineStr">
         <is>
           <t>任务</t>
         </is>
       </c>
-      <c r="E50" s="45" t="n"/>
-      <c r="F50" s="45" t="n"/>
-      <c r="G50" s="46" t="n"/>
+      <c r="E50" s="51" t="n"/>
+      <c r="F50" s="51" t="n"/>
+      <c r="G50" s="52" t="n"/>
       <c r="H50" s="32" t="n"/>
     </row>
     <row r="51" ht="22" customHeight="1" s="4">
@@ -2411,14 +2423,14 @@
           <t>1</t>
         </is>
       </c>
-      <c r="D51" s="48" t="inlineStr">
+      <c r="D51" s="38" t="inlineStr">
         <is>
           <t>回溯旧版模型分，作为新模型分的 baseline</t>
         </is>
       </c>
-      <c r="E51" s="45" t="n"/>
-      <c r="F51" s="45" t="n"/>
-      <c r="G51" s="46" t="n"/>
+      <c r="E51" s="51" t="n"/>
+      <c r="F51" s="51" t="n"/>
+      <c r="G51" s="52" t="n"/>
       <c r="H51" s="32" t="n"/>
     </row>
     <row r="52" ht="22" customHeight="1" s="4">
@@ -2429,14 +2441,14 @@
           <t>2</t>
         </is>
       </c>
-      <c r="D52" s="48" t="inlineStr">
+      <c r="D52" s="38" t="inlineStr">
         <is>
           <t>使用实验13248样本快速训练 Uplift 模型（S-learner / T-learner）</t>
         </is>
       </c>
-      <c r="E52" s="45" t="n"/>
-      <c r="F52" s="45" t="n"/>
-      <c r="G52" s="46" t="n"/>
+      <c r="E52" s="51" t="n"/>
+      <c r="F52" s="51" t="n"/>
+      <c r="G52" s="52" t="n"/>
       <c r="H52" s="32" t="n"/>
     </row>
     <row r="53">
@@ -2467,7 +2479,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="24" customHeight="1" s="4">
+    <row r="56" ht="22" customHeight="1" s="4">
       <c r="A56" s="32" t="n"/>
       <c r="B56" s="32" t="n"/>
       <c r="C56" s="39" t="inlineStr">
@@ -2490,12 +2502,13 @@
           <t>8月～9月</t>
         </is>
       </c>
-      <c r="G56" s="39" t="inlineStr">
+      <c r="G56" s="53" t="inlineStr">
         <is>
           <t>10月及以后</t>
         </is>
       </c>
-      <c r="H56" s="32" t="n"/>
+      <c r="H56" s="45" t="n"/>
+      <c r="I56" s="46" t="n"/>
     </row>
     <row r="57" ht="22" customHeight="1" s="4">
       <c r="A57" s="32" t="n"/>
@@ -2508,15 +2521,17 @@
       <c r="D57" s="45" t="n"/>
       <c r="E57" s="45" t="n"/>
       <c r="F57" s="45" t="n"/>
-      <c r="G57" s="46" t="n"/>
-      <c r="H57" s="32" t="n"/>
-    </row>
-    <row r="58" ht="20" customHeight="1" s="4">
+      <c r="G57" s="45" t="n"/>
+      <c r="H57" s="45" t="n"/>
+      <c r="I57" s="46" t="n"/>
+    </row>
+    <row r="58" ht="30" customHeight="1" s="4">
       <c r="A58" s="32" t="n"/>
       <c r="B58" s="32" t="n"/>
       <c r="C58" s="41" t="inlineStr">
         <is>
-          <t>• 启动方案2干净实验（15%+15%）</t>
+          <t>• 启动方案2干净实验
+（15%+15%）</t>
         </is>
       </c>
       <c r="D58" s="41" t="inlineStr">
@@ -2534,12 +2549,13 @@
           <t>• Qini/AUUC 监控</t>
         </is>
       </c>
-      <c r="G58" s="41" t="inlineStr">
+      <c r="G58" s="54" t="inlineStr">
         <is>
           <t>• 持续监控迭代</t>
         </is>
       </c>
-      <c r="H58" s="32" t="n"/>
+      <c r="H58" s="45" t="n"/>
+      <c r="I58" s="46" t="n"/>
     </row>
     <row r="59" ht="20" customHeight="1" s="4">
       <c r="A59" s="32" t="n"/>
@@ -2606,10 +2622,11 @@
           <t>阶段2：实时行为融合（实时打分服务）</t>
         </is>
       </c>
-      <c r="G62" s="46" t="n"/>
-      <c r="H62" s="32" t="n"/>
-    </row>
-    <row r="63" ht="20" customHeight="1" s="4">
+      <c r="G62" s="45" t="n"/>
+      <c r="H62" s="45" t="n"/>
+      <c r="I62" s="46" t="n"/>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="4">
       <c r="A63" s="32" t="n"/>
       <c r="B63" s="32" t="n"/>
       <c r="C63" s="32" t="n"/>
@@ -2620,12 +2637,13 @@
           <t>• 登录/还款实时特征接入</t>
         </is>
       </c>
-      <c r="G63" s="41" t="inlineStr">
+      <c r="G63" s="54" t="inlineStr">
         <is>
           <t>• 替换人工实时规则</t>
         </is>
       </c>
-      <c r="H63" s="32" t="n"/>
+      <c r="H63" s="45" t="n"/>
+      <c r="I63" s="46" t="n"/>
     </row>
     <row r="64" ht="20" customHeight="1" s="4">
       <c r="A64" s="32" t="n"/>
@@ -2658,12 +2676,13 @@
       <c r="D66" s="32" t="n"/>
       <c r="E66" s="32" t="n"/>
       <c r="F66" s="32" t="n"/>
-      <c r="G66" s="42" t="inlineStr">
+      <c r="G66" s="55" t="inlineStr">
         <is>
           <t>阶段3：素材选择模型（Contextual Bandit）</t>
         </is>
       </c>
-      <c r="H66" s="32" t="n"/>
+      <c r="H66" s="45" t="n"/>
+      <c r="I66" s="46" t="n"/>
     </row>
     <row r="67" ht="20" customHeight="1" s="4">
       <c r="A67" s="32" t="n"/>
@@ -2672,12 +2691,13 @@
       <c r="D67" s="32" t="n"/>
       <c r="E67" s="32" t="n"/>
       <c r="F67" s="32" t="n"/>
-      <c r="G67" s="41" t="inlineStr">
+      <c r="G67" s="54" t="inlineStr">
         <is>
           <t>• 素材特征工程</t>
         </is>
       </c>
-      <c r="H67" s="32" t="n"/>
+      <c r="H67" s="45" t="n"/>
+      <c r="I67" s="46" t="n"/>
     </row>
     <row r="68" ht="20" customHeight="1" s="4">
       <c r="A68" s="32" t="n"/>
@@ -2686,12 +2706,13 @@
       <c r="D68" s="32" t="n"/>
       <c r="E68" s="32" t="n"/>
       <c r="F68" s="32" t="n"/>
-      <c r="G68" s="41" t="inlineStr">
+      <c r="G68" s="54" t="inlineStr">
         <is>
           <t>• Bandit 模型上线</t>
         </is>
       </c>
-      <c r="H68" s="32" t="n"/>
+      <c r="H68" s="45" t="n"/>
+      <c r="I68" s="46" t="n"/>
     </row>
     <row r="69" ht="6" customHeight="1" s="4">
       <c r="A69" s="32" t="n"/>
@@ -2714,8 +2735,9 @@
           <t>阶段4：模型持续迭代与更新机制</t>
         </is>
       </c>
-      <c r="G70" s="46" t="n"/>
-      <c r="H70" s="32" t="n"/>
+      <c r="G70" s="45" t="n"/>
+      <c r="H70" s="45" t="n"/>
+      <c r="I70" s="46" t="n"/>
     </row>
     <row r="71" ht="20" customHeight="1" s="4">
       <c r="A71" s="32" t="n"/>
@@ -2728,12 +2750,13 @@
           <t>• 建立迭代流程规范</t>
         </is>
       </c>
-      <c r="G71" s="41" t="inlineStr">
+      <c r="G71" s="54" t="inlineStr">
         <is>
           <t>• 滚动重训</t>
         </is>
       </c>
-      <c r="H71" s="32" t="n"/>
+      <c r="H71" s="45" t="n"/>
+      <c r="I71" s="46" t="n"/>
     </row>
     <row r="72" ht="20" customHeight="1" s="4">
       <c r="A72" s="32" t="n"/>
@@ -2742,12 +2765,13 @@
       <c r="D72" s="32" t="n"/>
       <c r="E72" s="32" t="n"/>
       <c r="F72" s="32" t="n"/>
-      <c r="G72" s="41" t="inlineStr">
+      <c r="G72" s="54" t="inlineStr">
         <is>
           <t>• AB框架评估</t>
         </is>
       </c>
-      <c r="H72" s="32" t="n"/>
+      <c r="H72" s="45" t="n"/>
+      <c r="I72" s="46" t="n"/>
     </row>
     <row r="73" ht="6" customHeight="1" s="4">
       <c r="A73" s="32" t="n"/>
@@ -2803,25 +2827,27 @@
     <row r="79" ht="18" customHeight="1" s="4"/>
     <row r="80" ht="6" customHeight="1" s="4"/>
   </sheetData>
-  <mergeCells count="46">
+  <mergeCells count="53">
     <mergeCell ref="D18:G18"/>
     <mergeCell ref="C49:G49"/>
     <mergeCell ref="D9:G9"/>
     <mergeCell ref="C34:G34"/>
+    <mergeCell ref="G66:I66"/>
     <mergeCell ref="C24:G24"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="D25:G25"/>
     <mergeCell ref="C42:G42"/>
-    <mergeCell ref="B55:H55"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="D30:G30"/>
     <mergeCell ref="D15:G15"/>
-    <mergeCell ref="C3:G3"/>
     <mergeCell ref="D29:G29"/>
     <mergeCell ref="D51:G51"/>
     <mergeCell ref="B5:H5"/>
     <mergeCell ref="D38:G38"/>
+    <mergeCell ref="G68:I68"/>
     <mergeCell ref="D14:G14"/>
+    <mergeCell ref="C57:I57"/>
+    <mergeCell ref="G58:I58"/>
     <mergeCell ref="D26:G26"/>
     <mergeCell ref="B41:H41"/>
     <mergeCell ref="D35:G35"/>
@@ -2829,27 +2855,32 @@
     <mergeCell ref="D44:G44"/>
     <mergeCell ref="D10:G10"/>
     <mergeCell ref="C22:G22"/>
-    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="G63:I63"/>
     <mergeCell ref="D31:G31"/>
-    <mergeCell ref="F62:G62"/>
     <mergeCell ref="D45:G45"/>
     <mergeCell ref="D36:G36"/>
     <mergeCell ref="B21:H21"/>
     <mergeCell ref="D52:G52"/>
     <mergeCell ref="B48:H48"/>
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="D11:G11"/>
-    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="G56:I56"/>
     <mergeCell ref="D27:G27"/>
-    <mergeCell ref="G66"/>
+    <mergeCell ref="G72:I72"/>
     <mergeCell ref="D32:G32"/>
+    <mergeCell ref="G71:I71"/>
+    <mergeCell ref="C7:G7"/>
     <mergeCell ref="D17:G17"/>
-    <mergeCell ref="C7:G7"/>
+    <mergeCell ref="F70:I70"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="G67:I67"/>
     <mergeCell ref="D16:G16"/>
-    <mergeCell ref="C57:G57"/>
+    <mergeCell ref="F62:I62"/>
     <mergeCell ref="D43:G43"/>
     <mergeCell ref="C13:G13"/>
     <mergeCell ref="D37:G37"/>
     <mergeCell ref="D28:G28"/>
+    <mergeCell ref="C3:G3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>